<commit_message>
Add Hebrew translation layer, vendor inventory, and extended Mouser fields
Adds a central Hebrew translation dictionary for API lifecycle/status
strings, vendor-prefixed inventory display, and extraction of lead time,
unit price, suggested replacement, RoHS status, and packaging from Mouser
responses, surfaced as new columns in the GUI table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData.xlsx
+++ b/TestData.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\שלום\PycharmProjects\ShalomCI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aavi\ShalomCI\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50F0BBB-A54C-4A8C-A0E6-67077CAAD9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25125" windowHeight="12330"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -26,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
-    <t>UDN2987LW-6-T</t>
-  </si>
-  <si>
     <t>293D476X96R3B2TE3</t>
   </si>
   <si>
@@ -87,13 +85,16 @@
   </si>
   <si>
     <t>MPN</t>
+  </si>
+  <si>
+    <t>NE555P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,6 +109,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF303030"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -145,12 +151,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,156 +440,156 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="31.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:1">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:1">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:1">
+      <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+    <row r="15" spans="1:1">
+      <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+    <row r="16" spans="1:1" ht="15">
+      <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+    <row r="17" spans="1:1" ht="15">
+      <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+    <row r="18" spans="1:1" ht="15">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="19" spans="1:1" ht="15">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" ht="15">
       <c r="A20" s="2">
         <v>24070</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="30" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" ht="30">
       <c r="A21" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" ht="15">
       <c r="A23" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15">
+      <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+    <row r="25" spans="1:1" ht="15">
+      <c r="A25" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+    <row r="26" spans="1:1" ht="15">
+      <c r="A26" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" ht="15">
       <c r="A27" s="2">
         <v>24070</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="30" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1" ht="30">
       <c r="A28" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="15">
+      <c r="A29" s="3" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update sample BOM data; ignore Excel lock files and PyInstaller artifacts
- TestData.xlsx: refreshed sample BOM used for local testing (was
  sitting modified in the working tree across recent sessions).
- .gitignore: ignore ~$*.xlsx (Excel lock files created while a
  workbook is open) and PyInstaller outputs (build/, dist/, *.spec)
  that build.py generates - both kept reappearing as untracked noise
  and were being cleaned up manually every session.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData.xlsx
+++ b/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\aavi\ShalomCI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50F0BBB-A54C-4A8C-A0E6-67077CAAD9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6B9AEC-BEE6-48F8-ABDF-834593B0EA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-780" yWindow="2610" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>293D476X96R3B2TE3</t>
   </si>
@@ -36,27 +36,15 @@
     <t>STTHR106</t>
   </si>
   <si>
-    <t>1.5SMB33CA</t>
-  </si>
-  <si>
     <t>dspPIC33FJ256MC710-I/PF</t>
   </si>
   <si>
     <t>CR0805-FX33R0E</t>
   </si>
   <si>
-    <t>MMBT2222A/SOT</t>
-  </si>
-  <si>
-    <t>15UF/50V, 594D TENTA-R</t>
-  </si>
-  <si>
     <t>IRFPS3810</t>
   </si>
   <si>
-    <t>LM2676S-5.0/NOP</t>
-  </si>
-  <si>
     <t>B82789-C104</t>
   </si>
   <si>
@@ -66,28 +54,28 @@
     <t>293D475X9010A2T</t>
   </si>
   <si>
-    <t>CWROGKC225KC</t>
-  </si>
-  <si>
-    <t>222580500685K</t>
-  </si>
-  <si>
-    <t>LM193H/883B</t>
-  </si>
-  <si>
     <t>SARCON 200 XR-PE-200X300</t>
   </si>
   <si>
-    <t>WSL201OR5000FEA/195-C20438</t>
-  </si>
-  <si>
-    <t>10-497623-145</t>
-  </si>
-  <si>
     <t>MPN</t>
   </si>
   <si>
     <t>NE555P</t>
+  </si>
+  <si>
+    <t>CWR06KC225KC</t>
+  </si>
+  <si>
+    <t>WSL2010R5000FEA</t>
+  </si>
+  <si>
+    <t>37F2016D</t>
+  </si>
+  <si>
+    <t>NE555PWG4</t>
+  </si>
+  <si>
+    <t>NE555PWRG4</t>
   </si>
 </sst>
 </file>
@@ -111,9 +99,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="12"/>
       <color rgb="FF303030"/>
-      <name val="Arial Unicode MS"/>
+      <name val="Google Sans Text"/>
     </font>
   </fonts>
   <fills count="2">
@@ -151,16 +140,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="31.75" customWidth="1"/>
@@ -449,150 +438,123 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="A2" s="1"/>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A3" s="1"/>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="A4" s="1"/>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" spans="1:1">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
+      <c r="A9" s="6" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15">
-      <c r="A16" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="1"/>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="6"/>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" spans="1:1" ht="15">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15.75">
+      <c r="A22" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15.75">
+      <c r="A23" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15">
-      <c r="A17" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="15">
-      <c r="A18" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="15">
-      <c r="A19" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15">
-      <c r="A20" s="2">
-        <v>24070</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="30">
-      <c r="A21" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="15">
-      <c r="A22" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="15">
-      <c r="A23" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="15">
-      <c r="A24" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="15">
-      <c r="A25" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="15">
-      <c r="A26" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="15">
-      <c r="A27" s="2">
-        <v>24070</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="30">
-      <c r="A28" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="15">
-      <c r="A29" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A27">
+    <sortCondition ref="A1:A27"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>